<commit_message>
docs: set a wednesday deadline and fallback for the mentor data request
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BACKLOG.xlsx
+++ b/docs/BACKLOG.xlsx
@@ -248,16 +248,16 @@
     <t>W1-D6</t>
   </si>
   <si>
-    <t>Xin mentor file hóa đơn mẫu (tin nhắn đã soạn)</t>
+    <t>Xin mentor 2–3 file hóa đơn mẫu (đã nhắc lại, cho sẵn 3 lựa chọn). Hạn trả lời: thứ 4, 30/09/2026. Quá hạn hoặc bị từ chối → phương án B: dữ liệu sinh (W1-D1, W1-D2) và mẫu cào (W1-D4)</t>
   </si>
   <si>
     <t>Huy</t>
   </si>
   <si>
-    <t>3–4 file đại diện, hoặc 1 folder xuất hàng loạt</t>
-  </si>
-  <si>
-    <t>Có trả lời bằng văn bản; file thật chỉ để trên máy, không commit</t>
+    <t>2–3 file, hoặc mentor xác nhận dữ liệu sinh giống hóa đơn thật</t>
+  </si>
+  <si>
+    <t>Có trả lời bằng văn bản; file thật chỉ để trên máy, không commit. Không xóa dòng này — ghi kết quả vào báo cáo tuần</t>
   </si>
   <si>
     <t>P3</t>
@@ -4986,7 +4986,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C12A16CF-730C-4C76-995B-7EE67679F718}</x14:id>
+          <x14:id>{3D15D51A-3272-48A6-9EF1-CBD4BDD27861}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5042,7 +5042,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C12A16CF-730C-4C76-995B-7EE67679F718}">
+          <x14:cfRule type="dataBar" id="{3D15D51A-3272-48A6-9EF1-CBD4BDD27861}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5284,7 +5284,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{12749946-E308-4109-9F5C-AF0F33B5E254}</x14:id>
+          <x14:id>{D39ABB91-1B43-4963-944D-16CF50E9608D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5295,7 +5295,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{12749946-E308-4109-9F5C-AF0F33B5E254}">
+          <x14:cfRule type="dataBar" id="{D39ABB91-1B43-4963-944D-16CF50E9608D}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
docs: call the pilot company Doanh nghiệp X
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BACKLOG.xlsx
+++ b/docs/BACKLOG.xlsx
@@ -569,7 +569,7 @@
     <t>W1-C3</t>
   </si>
   <si>
-    <t>Nhóm thuế của các mặt hàng Xe X hay mua</t>
+    <t>Nhóm thuế của các mặt hàng Doanh nghiệp X hay mua</t>
   </si>
   <si>
     <t>Danh sách nhóm hàng → thuế suất, rà theo phụ lục nghị định</t>
@@ -644,7 +644,7 @@
     <t>U2</t>
   </si>
   <si>
-    <t>Chốt câu hỏi mở với mentor hoặc Xe X: Q1–Q6 trong USER_STORIES.md, đầu vào (một file nhiều hóa đơn? bảng kê?), dung sai, ngưỡng duyệt cấp 2, nhóm thuế của mặt hàng Xe X</t>
+    <t>Chốt câu hỏi mở với mentor hoặc Doanh nghiệp X: Q1–Q6 trong USER_STORIES.md, đầu vào (một file nhiều hóa đơn? bảng kê?), dung sai, ngưỡng duyệt cấp 2, nhóm thuế của mặt hàng Doanh nghiệp X</t>
   </si>
   <si>
     <t>Mỗi câu có quyết định và ngày chốt, ghi vào PRD</t>
@@ -4986,7 +4986,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3D15D51A-3272-48A6-9EF1-CBD4BDD27861}</x14:id>
+          <x14:id>{0B2304CC-DE7A-4CAD-A6BA-2BB9EC0BF64F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5042,7 +5042,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3D15D51A-3272-48A6-9EF1-CBD4BDD27861}">
+          <x14:cfRule type="dataBar" id="{0B2304CC-DE7A-4CAD-A6BA-2BB9EC0BF64F}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5284,7 +5284,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D39ABB91-1B43-4963-944D-16CF50E9608D}</x14:id>
+          <x14:id>{446D64F5-B823-42EE-9323-596125DD8C50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5295,7 +5295,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D39ABB91-1B43-4963-944D-16CF50E9608D}">
+          <x14:cfRule type="dataBar" id="{446D64F5-B823-42EE-9323-596125DD8C50}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
docs: call the pilot company Công ty X
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BACKLOG.xlsx
+++ b/docs/BACKLOG.xlsx
@@ -569,7 +569,7 @@
     <t>W1-C3</t>
   </si>
   <si>
-    <t>Nhóm thuế của các mặt hàng Doanh nghiệp X hay mua</t>
+    <t>Nhóm thuế của các mặt hàng Công ty X hay mua</t>
   </si>
   <si>
     <t>Danh sách nhóm hàng → thuế suất, rà theo phụ lục nghị định</t>
@@ -644,7 +644,7 @@
     <t>U2</t>
   </si>
   <si>
-    <t>Chốt câu hỏi mở với mentor hoặc Doanh nghiệp X: Q1–Q6 trong USER_STORIES.md, đầu vào (một file nhiều hóa đơn? bảng kê?), dung sai, ngưỡng duyệt cấp 2, nhóm thuế của mặt hàng Doanh nghiệp X</t>
+    <t>Chốt câu hỏi mở với mentor hoặc Công ty X: Q1–Q6 trong USER_STORIES.md, đầu vào (một file nhiều hóa đơn? bảng kê?), dung sai, ngưỡng duyệt cấp 2, nhóm thuế của mặt hàng Công ty X</t>
   </si>
   <si>
     <t>Mỗi câu có quyết định và ngày chốt, ghi vào PRD</t>
@@ -4986,7 +4986,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B2304CC-DE7A-4CAD-A6BA-2BB9EC0BF64F}</x14:id>
+          <x14:id>{212B76CC-483B-4320-B4D7-143F7F0B24A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5042,7 +5042,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B2304CC-DE7A-4CAD-A6BA-2BB9EC0BF64F}">
+          <x14:cfRule type="dataBar" id="{212B76CC-483B-4320-B4D7-143F7F0B24A2}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5284,7 +5284,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{446D64F5-B823-42EE-9323-596125DD8C50}</x14:id>
+          <x14:id>{33D6AB07-8852-4599-9422-195D04605FC8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5295,7 +5295,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{446D64F5-B823-42EE-9323-596125DD8C50}">
+          <x14:cfRule type="dataBar" id="{33D6AB07-8852-4599-9422-195D04605FC8}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
docs: the frontend is React and TypeScript from now on
The team moved straight to React with Vite on 30/09; the HTML prototype stays as the design reference and the no-install demo. F0 records the React scaffold on feat/frontend-react, F7 becomes porting the remaining screens.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BACKLOG.xlsx
+++ b/docs/BACKLOG.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="364">
   <si>
     <t>BACKLOG DỰ ÁN ĐỐI SOÁT HÓA ĐƠN — NHÓM FANTASTIC4</t>
   </si>
@@ -788,13 +788,28 @@
     <t>Có live URL cho giao diện</t>
   </si>
   <si>
+    <t>F0</t>
+  </si>
+  <si>
+    <t>Dựng khung React + TypeScript (Vite): đăng nhập, dashboard, danh sách hóa đơn</t>
+  </si>
+  <si>
+    <t>Có trên nhánh feat/frontend-react; chờ gộp vào nhánh chính</t>
+  </si>
+  <si>
+    <t>Giáp (gộp integ/mvp-rules trước)</t>
+  </si>
+  <si>
     <t>F7</t>
   </si>
   <si>
-    <t>Chuyển giao diện sang React, dùng lại module gọi API và bộ màu</t>
-  </si>
-  <si>
-    <t>Chạy đủ kịch bản demo như bản HTML</t>
+    <t>Chuyển nốt các màn còn lại từ prototype sang React: so sánh ba chiều, ngoại lệ, tóm tắt duyệt, hàng đợi duyệt, NCC, cấu hình</t>
+  </si>
+  <si>
+    <t>3–4</t>
+  </si>
+  <si>
+    <t>Chạy đủ kịch bản demo 5 phút như bản prototype</t>
   </si>
   <si>
     <t>Đổi tab Bút toán trong prototype thành Tóm tắt duyệt; trạng thái cuối là Đã xuất cho kế toán (PRD F10, WIREFRAME S7)</t>
@@ -858,9 +873,6 @@
   </si>
   <si>
     <t>Độ tin cậy từng trường và hiệu chỉnh ngưỡng trên bộ đánh giá</t>
-  </si>
-  <si>
-    <t>3–4</t>
   </si>
   <si>
     <t>Ngưỡng do dữ liệu chọn; sai mà không gắn cờ ≈ 0</t>
@@ -3677,13 +3689,13 @@
         <v>78</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>26</v>
+        <v>206</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H18" s="25">
         <v>0</v>
@@ -3693,7 +3705,7 @@
         <v>259</v>
       </c>
       <c r="K18" s="20" t="s">
-        <v>1</v>
+        <v>260</v>
       </c>
       <c r="L18" s="24"/>
       <c r="M18" s="24"/>
@@ -3701,19 +3713,19 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
-        <v>116</v>
+        <v>261</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>239</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>78</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>241</v>
+        <v>263</v>
       </c>
       <c r="F19" s="21" t="s">
         <v>22</v>
@@ -3726,7 +3738,7 @@
       </c>
       <c r="I19" s="26"/>
       <c r="J19" s="20" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="K19" s="20" t="s">
         <v>1</v>
@@ -3737,19 +3749,19 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>206</v>
+        <v>241</v>
       </c>
       <c r="F20" s="21" t="s">
         <v>22</v>
@@ -3762,10 +3774,10 @@
       </c>
       <c r="I20" s="26"/>
       <c r="J20" s="20" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K20" s="20" t="s">
-        <v>265</v>
+        <v>1</v>
       </c>
       <c r="L20" s="24"/>
       <c r="M20" s="24"/>
@@ -3773,13 +3785,13 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>160</v>
+        <v>93</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>63</v>
@@ -3798,10 +3810,10 @@
       </c>
       <c r="I21" s="26"/>
       <c r="J21" s="20" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="K21" s="20" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="L21" s="24"/>
       <c r="M21" s="24"/>
@@ -3809,13 +3821,13 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>269</v>
+        <v>160</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>63</v>
@@ -3834,10 +3846,10 @@
       </c>
       <c r="I22" s="26"/>
       <c r="J22" s="20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K22" s="20" t="s">
-        <v>1</v>
+        <v>273</v>
       </c>
       <c r="L22" s="24"/>
       <c r="M22" s="24"/>
@@ -3845,19 +3857,19 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D23" s="21" t="s">
         <v>63</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>241</v>
+        <v>206</v>
       </c>
       <c r="F23" s="21" t="s">
         <v>22</v>
@@ -3870,7 +3882,7 @@
       </c>
       <c r="I23" s="26"/>
       <c r="J23" s="20" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="K23" s="20" t="s">
         <v>1</v>
@@ -3881,13 +3893,13 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>63</v>
@@ -3906,10 +3918,10 @@
       </c>
       <c r="I24" s="26"/>
       <c r="J24" s="20" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="K24" s="20" t="s">
-        <v>278</v>
+        <v>1</v>
       </c>
       <c r="L24" s="24"/>
       <c r="M24" s="24"/>
@@ -3917,19 +3929,19 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>63</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>281</v>
+        <v>241</v>
       </c>
       <c r="F25" s="21" t="s">
         <v>22</v>
@@ -3945,7 +3957,7 @@
         <v>282</v>
       </c>
       <c r="K25" s="20" t="s">
-        <v>1</v>
+        <v>283</v>
       </c>
       <c r="L25" s="24"/>
       <c r="M25" s="24"/>
@@ -3953,19 +3965,19 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>63</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>213</v>
+        <v>263</v>
       </c>
       <c r="F26" s="21" t="s">
         <v>22</v>
@@ -3978,7 +3990,7 @@
       </c>
       <c r="I26" s="26"/>
       <c r="J26" s="20" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K26" s="20" t="s">
         <v>1</v>
@@ -3989,19 +4001,19 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
-        <v>66</v>
+        <v>287</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>63</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>287</v>
+        <v>213</v>
       </c>
       <c r="F27" s="21" t="s">
         <v>22</v>
@@ -4014,10 +4026,10 @@
       </c>
       <c r="I27" s="26"/>
       <c r="J27" s="20" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K27" s="20" t="s">
-        <v>289</v>
+        <v>1</v>
       </c>
       <c r="L27" s="24"/>
       <c r="M27" s="24"/>
@@ -4025,22 +4037,22 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>267</v>
+      </c>
+      <c r="C28" s="20" t="s">
         <v>290</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>262</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>291</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>63</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>26</v>
+        <v>291</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G28" s="23" t="s">
         <v>11</v>
@@ -4061,22 +4073,22 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>56</v>
+        <v>294</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>294</v>
+        <v>267</v>
       </c>
       <c r="C29" s="20" t="s">
         <v>295</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>206</v>
+        <v>26</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G29" s="23" t="s">
         <v>11</v>
@@ -4089,7 +4101,7 @@
         <v>296</v>
       </c>
       <c r="K29" s="20" t="s">
-        <v>1</v>
+        <v>297</v>
       </c>
       <c r="L29" s="24"/>
       <c r="M29" s="24"/>
@@ -4097,13 +4109,13 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>53</v>
@@ -4122,7 +4134,7 @@
       </c>
       <c r="I30" s="26"/>
       <c r="J30" s="20" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="K30" s="20" t="s">
         <v>1</v>
@@ -4133,19 +4145,19 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>53</v>
       </c>
       <c r="E31" s="21" t="s">
-        <v>287</v>
+        <v>206</v>
       </c>
       <c r="F31" s="21" t="s">
         <v>22</v>
@@ -4158,10 +4170,10 @@
       </c>
       <c r="I31" s="26"/>
       <c r="J31" s="20" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="K31" s="20" t="s">
-        <v>301</v>
+        <v>1</v>
       </c>
       <c r="L31" s="24"/>
       <c r="M31" s="24"/>
@@ -4169,10 +4181,10 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="18" t="s">
-        <v>302</v>
+        <v>109</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C32" s="20" t="s">
         <v>303</v>
@@ -4181,7 +4193,7 @@
         <v>53</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>241</v>
+        <v>291</v>
       </c>
       <c r="F32" s="21" t="s">
         <v>22</v>
@@ -4197,7 +4209,7 @@
         <v>304</v>
       </c>
       <c r="K32" s="20" t="s">
-        <v>268</v>
+        <v>305</v>
       </c>
       <c r="L32" s="24"/>
       <c r="M32" s="24"/>
@@ -4205,13 +4217,13 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D33" s="21" t="s">
         <v>53</v>
@@ -4230,10 +4242,10 @@
       </c>
       <c r="I33" s="26"/>
       <c r="J33" s="20" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K33" s="20" t="s">
-        <v>308</v>
+        <v>273</v>
       </c>
       <c r="L33" s="24"/>
       <c r="M33" s="24"/>
@@ -4244,7 +4256,7 @@
         <v>309</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C34" s="20" t="s">
         <v>310</v>
@@ -4269,7 +4281,7 @@
         <v>311</v>
       </c>
       <c r="K34" s="20" t="s">
-        <v>1</v>
+        <v>312</v>
       </c>
       <c r="L34" s="24"/>
       <c r="M34" s="24"/>
@@ -4277,22 +4289,22 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D35" s="21" t="s">
         <v>53</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="F35" s="21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G35" s="23" t="s">
         <v>11</v>
@@ -4302,10 +4314,10 @@
       </c>
       <c r="I35" s="26"/>
       <c r="J35" s="20" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K35" s="20" t="s">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="L35" s="24"/>
       <c r="M35" s="24"/>
@@ -4313,13 +4325,13 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D36" s="21" t="s">
         <v>53</v>
@@ -4338,10 +4350,10 @@
       </c>
       <c r="I36" s="26"/>
       <c r="J36" s="20" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K36" s="20" t="s">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="L36" s="24"/>
       <c r="M36" s="24"/>
@@ -4349,22 +4361,22 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D37" s="21" t="s">
         <v>53</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>26</v>
+        <v>213</v>
       </c>
       <c r="F37" s="21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G37" s="23" t="s">
         <v>11</v>
@@ -4374,7 +4386,7 @@
       </c>
       <c r="I37" s="26"/>
       <c r="J37" s="20" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K37" s="20" t="s">
         <v>1</v>
@@ -4385,22 +4397,22 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
-        <v>141</v>
+        <v>322</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>321</v>
+        <v>298</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>206</v>
+        <v>26</v>
       </c>
       <c r="F38" s="21" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G38" s="23" t="s">
         <v>11</v>
@@ -4410,10 +4422,10 @@
       </c>
       <c r="I38" s="26"/>
       <c r="J38" s="20" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K38" s="20" t="s">
-        <v>324</v>
+        <v>1</v>
       </c>
       <c r="L38" s="24"/>
       <c r="M38" s="24"/>
@@ -4421,13 +4433,13 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>143</v>
+        <v>326</v>
       </c>
       <c r="D39" s="21" t="s">
         <v>96</v>
@@ -4446,10 +4458,10 @@
       </c>
       <c r="I39" s="26"/>
       <c r="J39" s="20" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="K39" s="20" t="s">
-        <v>1</v>
+        <v>328</v>
       </c>
       <c r="L39" s="24"/>
       <c r="M39" s="24"/>
@@ -4457,19 +4469,19 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>326</v>
+        <v>143</v>
       </c>
       <c r="D40" s="21" t="s">
         <v>96</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>287</v>
+        <v>206</v>
       </c>
       <c r="F40" s="21" t="s">
         <v>22</v>
@@ -4482,7 +4494,7 @@
       </c>
       <c r="I40" s="26"/>
       <c r="J40" s="20" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="K40" s="20" t="s">
         <v>1</v>
@@ -4493,19 +4505,19 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="18" t="s">
-        <v>328</v>
+        <v>151</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D41" s="21" t="s">
         <v>96</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>241</v>
+        <v>291</v>
       </c>
       <c r="F41" s="21" t="s">
         <v>22</v>
@@ -4518,7 +4530,7 @@
       </c>
       <c r="I41" s="26"/>
       <c r="J41" s="20" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="K41" s="20" t="s">
         <v>1</v>
@@ -4529,13 +4541,13 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
-        <v>99</v>
+        <v>332</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D42" s="21" t="s">
         <v>96</v>
@@ -4554,7 +4566,7 @@
       </c>
       <c r="I42" s="26"/>
       <c r="J42" s="20" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="K42" s="20" t="s">
         <v>1</v>
@@ -4565,13 +4577,13 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="18" t="s">
-        <v>333</v>
+        <v>99</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D43" s="21" t="s">
         <v>96</v>
@@ -4590,7 +4602,7 @@
       </c>
       <c r="I43" s="26"/>
       <c r="J43" s="20" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K43" s="20" t="s">
         <v>1</v>
@@ -4601,13 +4613,13 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D44" s="21" t="s">
         <v>96</v>
@@ -4626,10 +4638,10 @@
       </c>
       <c r="I44" s="26"/>
       <c r="J44" s="20" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K44" s="20" t="s">
-        <v>324</v>
+        <v>1</v>
       </c>
       <c r="L44" s="24"/>
       <c r="M44" s="24"/>
@@ -4637,19 +4649,19 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="18" t="s">
-        <v>170</v>
+        <v>340</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D45" s="21" t="s">
         <v>96</v>
       </c>
       <c r="E45" s="21" t="s">
-        <v>340</v>
+        <v>241</v>
       </c>
       <c r="F45" s="21" t="s">
         <v>22</v>
@@ -4662,10 +4674,10 @@
       </c>
       <c r="I45" s="26"/>
       <c r="J45" s="20" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K45" s="20" t="s">
-        <v>1</v>
+        <v>328</v>
       </c>
       <c r="L45" s="24"/>
       <c r="M45" s="24"/>
@@ -4673,19 +4685,19 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D46" s="21" t="s">
         <v>96</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>241</v>
+        <v>344</v>
       </c>
       <c r="F46" s="21" t="s">
         <v>22</v>
@@ -4698,7 +4710,7 @@
       </c>
       <c r="I46" s="26"/>
       <c r="J46" s="20" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="K46" s="20" t="s">
         <v>1</v>
@@ -4707,7 +4719,42 @@
       <c r="M46" s="24"/>
       <c r="N46" s="26"/>
     </row>
-    <row r="47" spans="4:14" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>325</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>346</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="E47" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="F47" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="G47" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" s="25">
+        <v>0</v>
+      </c>
+      <c r="I47" s="26"/>
+      <c r="J47" s="20" t="s">
+        <v>347</v>
+      </c>
+      <c r="K47" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="L47" s="24"/>
+      <c r="M47" s="24"/>
+      <c r="N47" s="26"/>
+    </row>
     <row r="48" spans="4:14" x14ac:dyDescent="0.25"/>
     <row r="49" spans="4:14" x14ac:dyDescent="0.25"/>
     <row r="50" spans="4:14" x14ac:dyDescent="0.25"/>
@@ -4962,7 +5009,7 @@
     <row r="299" spans="4:14" x14ac:dyDescent="0.25"/>
     <row r="300" spans="4:14" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:N46"/>
+  <autoFilter ref="A1:N47"/>
   <conditionalFormatting sqref="G2:G300">
     <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"Đang làm"</formula>
@@ -4986,7 +5033,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{212B76CC-483B-4320-B4D7-143F7F0B24A2}</x14:id>
+          <x14:id>{A0D9AAAC-EE6B-4884-8FFF-29A87A07E372}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5042,7 +5089,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{212B76CC-483B-4320-B4D7-143F7F0B24A2}">
+          <x14:cfRule type="dataBar" id="{A0D9AAAC-EE6B-4884-8FFF-29A87A07E372}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5077,17 +5124,17 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>11</v>
@@ -5105,13 +5152,13 @@
         <v>19</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -5261,7 +5308,7 @@
     </row>
     <row r="11" spans="1:1" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -5284,7 +5331,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{33D6AB07-8852-4599-9422-195D04605FC8}</x14:id>
+          <x14:id>{C7D62D37-2F02-4B68-836F-17AE08F4BF83}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5295,7 +5342,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{33D6AB07-8852-4599-9422-195D04605FC8}">
+          <x14:cfRule type="dataBar" id="{C7D62D37-2F02-4B68-836F-17AE08F4BF83}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5332,19 +5379,19 @@
         <v>194</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -5355,16 +5402,16 @@
         <v>46291.70833333333</v>
       </c>
       <c r="C2" s="36" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="D2" s="36" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="F2" s="36" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>